<commit_message>
docs(topic-13): update README difficulty + references spreadsheet
README.md: Topic 13 difficulty label 'Foundational' → 'Intermediate'
to match the planning-document decision (track-opener topics at this
depth are calibrated intermediate — same as Topics 9 and 12).

docs/formalstatistics-citations.xlsx:
- Added 3 new citations: LEH1998 (Lehmann & Casella, Theory of Point
  Estimation), BIC2015 (Bickel & Doksum, Mathematical Statistics),
  STE1956 (Stein, inadmissibility of the sample mean — the original
  James-Stein paper).
- Populated HAS2009 (Hastie, Tibshirani & Friedman, ESL) previously
  empty row with full metadata and point-estimation usage.
- Appended point-estimation to Used-In-Topics for 4 existing refs:
  BIL2012, WAS2004, BIS2006, CAS2002.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalstatistics-citations.xlsx
+++ b/docs/formalstatistics-citations.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -562,7 +562,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>sample-spaces, conditional-probability, random-variables, large-deviations</t>
+          <t>sample-spaces, conditional-probability, random-variables, large-deviations, point-estimation</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>sample-spaces, conditional-probability, random-variables, large-deviations</t>
+          <t>sample-spaces, conditional-probability, random-variables, large-deviations, point-estimation</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>conditional-probability, random-variables, large-deviations</t>
+          <t>conditional-probability, random-variables, large-deviations, point-estimation</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>random-variables, large-deviations</t>
+          <t>random-variables, large-deviations, point-estimation</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1074,6 +1074,21 @@
           <t>https://hastie.su.domains/ElemStatLearn/</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>point-estimation</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Ch 7.3: bias-variance decomposition for prediction error — the ML version of the MSE decomposition</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1310,6 +1325,161 @@
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Standard graduate reference for large deviations theory; Cramér, Sanov, Varadhan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LEH1998</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Erich L. Lehmann &amp; George Casella</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Theory of Point Estimation</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1998</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>978-0-387-98502-2</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/book/10.1007/b98854</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>point-estimation</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Definitive graduate-level reference on point estimation. Ch 1-2 cover unbiasedness, MSE, and the CRLB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BIC2015</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Peter J. Bickel &amp; Kjell A. Doksum</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mathematical Statistics: Basic Ideas and Selected Topics</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>CRC Press</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>978-1-498-72380-0</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.routledge.com/Mathematical-Statistics-Basic-Ideas-and-Selected-Topics-Volume-I/Bickel-Doksum/p/book/9781498723800</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>point-estimation</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Ch 3: Fisher information, score function, CRLB with careful regularity-condition exposition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>STE1956</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Charles Stein</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Inadmissibility of the Usual Estimator for the Mean of a Multivariate Normal Distribution</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1956</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Proceedings of the Third Berkeley Symposium</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://projecteuclid.org/euclid.bsmsp/1200501656</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>point-estimation</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Vol 1, pp 197-206. Original proof that the sample mean is inadmissible in dimension d &gt;= 3. Foundation of shrinkage estimation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Merge pull request #15 from jonx0037/topic-14/maximum-likelihood"
This reverts commit 8ed54ce21db456ea1ef51e1f12dd0f70ceba8f7f, reversing
changes made to 1523f02e1b369c17dbcb8bcdea82698a49e02d58.
</commit_message>
<xml_diff>
--- a/docs/formalstatistics-citations.xlsx
+++ b/docs/formalstatistics-citations.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -723,7 +723,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>sample-spaces, conditional-probability, random-variables, large-deviations, point-estimation, maximum-likelihood</t>
+          <t>sample-spaces, conditional-probability, random-variables, large-deviations, point-estimation</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>conditional-probability, random-variables, large-deviations, point-estimation, maximum-likelihood</t>
+          <t>conditional-probability, random-variables, large-deviations, point-estimation</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>random-variables, large-deviations, point-estimation, maximum-likelihood</t>
+          <t>random-variables, large-deviations, point-estimation</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>point-estimation, maximum-likelihood</t>
+          <t>point-estimation</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>point-estimation, maximum-likelihood</t>
+          <t>point-estimation</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1480,116 +1480,6 @@
       <c r="K20" t="inlineStr">
         <is>
           <t>Vol 1, pp 197-206. Original proof that the sample mean is inadmissible in dimension d &gt;= 3. Foundation of shrinkage estimation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>VDV1998</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>A. W. van der Vaart</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Asymptotic Statistics</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>1998</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Cambridge University Press</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>978-0-521-78450-4</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>https://www.cambridge.org/core/books/asymptotic-statistics/A3C7DAD3F7E66A1FA60E9C8FE132EE1D</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Book</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>maximum-likelihood</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Chapter 5 (M-Estimators and Maximum Likelihood) gives the modern treatment of MLE asymptotics. Theorem 5.39 is the asymptotic-normality result followed in Topic 14 §14.5.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>NOC2006</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Jorge Nocedal &amp; Stephen J. Wright</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Numerical Optimization</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>2006</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Springer</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>978-0-387-30303-1</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>https://link.springer.com/book/10.1007/978-0-387-40065-5</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Book</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>maximum-likelihood</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Chapter 2 covers Newton's method and quadratic convergence theory; Chapter 11 treats Fisher scoring and related maximum-likelihood iterations. Used in Topic 14 §14.7.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reapply "Merge pull request #15 from jonx0037/topic-14/maximum-likelihood"
This reverts commit 58da0a1303896cc5e5cb55a070dcf965c292f057.
</commit_message>
<xml_diff>
--- a/docs/formalstatistics-citations.xlsx
+++ b/docs/formalstatistics-citations.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -723,7 +723,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>sample-spaces, conditional-probability, random-variables, large-deviations, point-estimation</t>
+          <t>sample-spaces, conditional-probability, random-variables, large-deviations, point-estimation, maximum-likelihood</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>conditional-probability, random-variables, large-deviations, point-estimation</t>
+          <t>conditional-probability, random-variables, large-deviations, point-estimation, maximum-likelihood</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>random-variables, large-deviations, point-estimation</t>
+          <t>random-variables, large-deviations, point-estimation, maximum-likelihood</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>point-estimation</t>
+          <t>point-estimation, maximum-likelihood</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>point-estimation</t>
+          <t>point-estimation, maximum-likelihood</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1480,6 +1480,116 @@
       <c r="K20" t="inlineStr">
         <is>
           <t>Vol 1, pp 197-206. Original proof that the sample mean is inadmissible in dimension d &gt;= 3. Foundation of shrinkage estimation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>VDV1998</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>A. W. van der Vaart</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Asymptotic Statistics</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1998</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Cambridge University Press</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>978-0-521-78450-4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.cambridge.org/core/books/asymptotic-statistics/A3C7DAD3F7E66A1FA60E9C8FE132EE1D</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>maximum-likelihood</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Chapter 5 (M-Estimators and Maximum Likelihood) gives the modern treatment of MLE asymptotics. Theorem 5.39 is the asymptotic-normality result followed in Topic 14 §14.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NOC2006</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Jorge Nocedal &amp; Stephen J. Wright</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Numerical Optimization</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>978-0-387-30303-1</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/book/10.1007/978-0-387-40065-5</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>maximum-likelihood</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Chapter 2 covers Newton's method and quadratic convergence theory; Chapter 11 treats Fisher scoring and related maximum-likelihood iterations. Used in Topic 14 §14.7.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(citations): +10 entries for Topic 28; +4 slug appends
Brief §8.4 updates to the references spreadsheet:

  New rows (10): JAM1961, EFR1973, LIN1972, LAI1982, GEL2006, HAR1977,
  BRO2003, RUB1981, BET2015, KLE2012 — full Chicago-ish formatting,
  all URLs verified.

  Slug appends to "Used In Topics" column (4): STE1956, NEA2011,
  GEL2013, LEH1998 — added hierarchical-bayes-and-partial-pooling to
  each. Note: the spreadsheet uses topic slugs (not numbers) for this
  column, so the appends are slug-form rather than "28".

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalstatistics-citations.xlsx
+++ b/docs/formalstatistics-citations.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>point-estimation, maximum-likelihood, method-of-moments, sufficient-statistics</t>
+          <t>point-estimation, maximum-likelihood, method-of-moments, sufficient-statistics, hierarchical-bayes-and-partial-pooling</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>point-estimation, regularization-and-penalized-estimation</t>
+          <t>point-estimation, regularization-and-penalized-estimation, hierarchical-bayes-and-partial-pooling</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>hypothesis-testing, bayesian-computation-and-mcmc, bayesian-model-comparison-and-bma</t>
+          <t>hypothesis-testing, bayesian-computation-and-mcmc, bayesian-model-comparison-and-bma, hierarchical-bayes-and-partial-pooling</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -4606,7 +4606,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>bayesian-computation-and-mcmc</t>
+          <t>bayesian-computation-and-mcmc, hierarchical-bayes-and-partial-pooling</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -5417,6 +5417,456 @@
       <c r="K105" t="inlineStr">
         <is>
           <t>Origin of Bayesian posterior-predictive p-value p_B (§27.9 Ex 12).</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>JAM1961</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Willard James, Charles Stein</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Estimation with Quadratic Loss</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>1961</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Proceedings of the Fourth Berkeley Symposium on Mathematical Statistics and Probability, vol. 1, pp. 361–379</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>https://projecteuclid.org/ebooks/berkeley-symposium-on-mathematical-statistics-and-probability/Proceedings-of-the-Fourth-Berkeley-Symposium-on-Mathematical-Statistics-and/chapter/Estimation-with-Quadratic-Loss/bsmsp/1200512173</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>James–Stein estimator + closed-form risk dominance result. Used in §28.5 Thm 2 and Proof 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>EFR1973</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Bradley Efron, Carl Morris</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Stein's Estimation Rule and Its Competitors — an Empirical Bayes Approach</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>1973</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Journal of the American Statistical Association, 68(341), pp. 117–130</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>https://www.jstor.org/stable/2284155</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Positive-part JS (§28.5 Rem 11) and empirical-Bayes rereading of shrinkage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>LIN1972</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Dennis V. Lindley, Adrian F. M. Smith</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Bayes Estimates for the Linear Model</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>1972</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Journal of the Royal Statistical Society: Series B, 34(1), pp. 1–41</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>https://www.jstor.org/stable/2985048</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Origin of Bayesian partial pooling in hierarchical linear models (§28.6 Rem 13).</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>LAI1982</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Nan M. Laird, James H. Ware</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Random-Effects Models for Longitudinal Data</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>1982</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Biometrics, 38(4), pp. 963–974</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>https://www.jstor.org/stable/2529876</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Canonical linear mixed-effects model (§28.8 Def 5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>GEL2006</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Andrew Gelman</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Prior Distributions for Variance Parameters in Hierarchical Models</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>2006</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Bayesian Analysis, 1(3), pp. 515–534</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>https://projecteuclid.org/journals/bayesian-analysis/volume-1/issue-3/Prior-distributions-for-variance-parameters-in-hierarchical-models-comment-on/10.1214/06-BA117A.full</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Half-Cauchy hyperpriors on τ — modern default (§28.7 Rem 17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>HAR1977</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>David A. Harville</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Maximum Likelihood Approaches to Variance Component Estimation and to Related Problems</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>1977</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Journal of the American Statistical Association, 72(358), pp. 320–338</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>https://www.jstor.org/stable/2286796</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>REML as frequentist-mixed-models companion (§28.8 Rem 20).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>BRO2003</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>William J. Browne, David Draper</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>A Comparison of Bayesian and Likelihood-Based Methods for Fitting Multilevel Models</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>2006</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Bayesian Analysis, 1(3), pp. 473–514</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>https://projecteuclid.org/journals/bayesian-analysis/volume-1/issue-3/A-comparison-of-Bayesian-and-likelihood-based-methods-for-fitting/10.1214/06-BA117.full</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Head-to-head Bayesian vs likelihood multilevel methods (§28.8 background).</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>RUB1981</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Donald B. Rubin</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Estimation in Parallel Randomized Experiments</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>1981</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Journal of Educational Statistics, 6(4), pp. 377–401</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>https://www.jstor.org/stable/1164617</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>8-schools dataset — spine example across §§28.1/28.4/28.6/28.9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>BET2015</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Michael Betancourt, Mark Girolami</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Hamiltonian Monte Carlo for Hierarchical Models</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>2015</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Current Trends in Bayesian Methodology with Applications (Chapman &amp; Hall/CRC), pp. 79–101</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/1312.0906</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Chapter</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>§3 develops funnel-geometry analysis cited in §28.9 Thm 7 Proof 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>KLE2012</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Bas J. K. Kleijn, Aad W. van der Vaart</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>The Bernstein–Von Mises Theorem under Misspecification</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>2012</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Electronic Journal of Statistics, 6, pp. 354–381</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>https://projecteuclid.org/journals/electronic-journal-of-statistics/volume-6/issue-none/The-Bernstein-Von-Mises-theorem-under-misspecification/10.1214/12-EJS675.full</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>hierarchical-bayes-and-partial-pooling</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>BvM under misspecification; cited in §28.7 Thm 5 as the Type-II MLE consistency source.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(topic-30): Kernel Density Estimation (Track 8, 2/4)
Discharges:
- Topic 7 §7.13 "coming soon" KDE promise (continuous-distributions.mdx:917)
- Topic 29 §29.6 Rem 12 density-at-quantile pointer (order-statistics-and-quantiles.mdx:590)

Contents:
- 10 sections, 7 theorems (1 full + 1 short + 1 sketched + 4 stated), 13 examples, 22 remarks
- 9 figures, 3 required + 1 optional interactive components (BandwidthExplorer featured)
- 13 new shared-module exports in nonparametric.ts §§8-12, 14 new test pins (T30.1-T30.14)
- 9 new citations (ROS1956, PAR1962, EPA1969, SIL1986, SHJ1991, WAN1995, FAN1996, DUO2007, SCO2015) + 3 reused-row appends (VDV1998, SER1980, LEH1998)
- 5 cross-reference edits (E1-E5): continuous-distributions.mdx, order-statistics-and-quantiles.mdx x3, linear-regression.mdx

Featured: §30.6 AMISE decomposition + optimal h* (full proof); Epanechnikov optimality (short proof).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalstatistics-citations.xlsx
+++ b/docs/formalstatistics-citations.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="640" windowWidth="34560" windowHeight="21700" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Citations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Citations" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Citations'!$A$1:$K$8</definedName>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K125"/>
+  <dimension ref="A1:K134"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>point-estimation, maximum-likelihood, method-of-moments, sufficient-statistics, hierarchical-bayes-and-partial-pooling, order-statistics-and-quantiles</t>
+          <t>point-estimation, maximum-likelihood, method-of-moments, sufficient-statistics, hierarchical-bayes-and-partial-pooling, order-statistics-and-quantiles, kernel-density-estimation</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>maximum-likelihood, method-of-moments, bayesian-computation-and-mcmc, order-statistics-and-quantiles</t>
+          <t>maximum-likelihood, method-of-moments, bayesian-computation-and-mcmc, order-statistics-and-quantiles, kernel-density-estimation</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -6321,12 +6321,442 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>central-limit-theorem, point-estimation, order-statistics-and-quantiles</t>
+          <t>central-limit-theorem, point-estimation, order-statistics-and-quantiles, kernel-density-estimation</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
           <t>§2.3 on order statistics; §2.5 on quantile functions (Bahadur proof citation); §2.4 on the ECDF. Referenced by Topic 29 §29.6 Proof 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>ROS1956</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Murray Rosenblatt</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Remarks on Some Nonparametric Estimates of a Density Function</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>1956</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Annals of Mathematical Statistics 27(3): 832–837</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>https://projecteuclid.org/journals/annals-of-mathematical-statistics/volume-27/issue-3/Remarks-on-Some-Nonparametric-Estimates-of-a-Density-Function/10.1214/aoms/1177728190.full</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>kernel-density-estimation</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>The founding paper of kernel smoothing. Bias-variance framework; bias is O(h²) under regularity. §30.4 Rem 7 Rosenblatt no-free-lunch attribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>PAR1962</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Emanuel Parzen</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>On Estimation of a Probability Density Function and Mode</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>1962</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Annals of Mathematical Statistics 33(3): 1065–1076</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>https://projecteuclid.org/journals/annals-of-mathematical-statistics/volume-33/issue-3/On-Estimation-of-a-Probability-Density-Function-and-Mode/10.1214/aoms/1177704472.full</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>kernel-density-estimation</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Generalizes Rosenblatt to arbitrary symmetric kernels; proves pointwise asymptotic normality. §30.7 Thm 6 Parzen's theorem attribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>EPA1969</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Vassiliy A. Epanechnikov</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Non-Parametric Estimation of a Multivariate Probability Density</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>1969</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Theory of Probability &amp; Its Applications 14(1): 153–158</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>https://epubs.siam.org/doi/10.1137/1114019</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>kernel-density-estimation</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Proves the MISE-optimal kernel is K_E(u) = (3/4)(1 − u²) 1{|u| ≤ 1}. §30.6 Thm 5 Epanechnikov optimality short-proof attribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>SIL1986</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Bernard W. Silverman</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Density Estimation for Statistics and Data Analysis</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>1986</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Chapman and Hall</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>978-0-412-24620-3</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>https://www.taylorfrancis.com/books/mono/10.1201/9781315140919/density-estimation-statistics-data-analysis-bernard-silverman</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>kernel-density-estimation</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Standard monograph on univariate KDE. §3.4 derives ĥ_ROT = 1.06 σ̂ n^(−1/5) (and the robust min(σ̂, IQR/1.34) variant) used in §30.8 Thm 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>SHJ1991</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Simon J. Sheather, M. Chris Jones</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>A Reliable Data-Based Bandwidth Selection Method for Kernel Density Estimation</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>1991</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Journal of the Royal Statistical Society: Series B (Methodological) 53(3): 683–690</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/j.2517-6161.1991.tb01857.x</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>kernel-density-estimation</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>The plug-in bandwidth selector — gold standard. §30.8 Thm 7 name-check; §30.8 Ex 10 + PluginBandwidthComparator component benchmark against SHJ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>WAN1995</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>M. P. Wand, M. C. Jones</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Kernel Smoothing</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>1995</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Chapman and Hall/CRC</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>978-0-412-55270-0</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>https://www.taylorfrancis.com/books/mono/10.1201/b14876/kernel-smoothing-wand-jones</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>kernel-density-estimation</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Modern monograph. §2.5 has the MISE/AMISE development (§30.5–§30.6); §3 has the bandwidth-selection catalog (§30.8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>FAN1996</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Jianqing Fan, Irène Gijbels</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Local Polynomial Modelling and Its Applications</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>1996</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Chapman and Hall/CRC</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>978-0-412-98321-4</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>https://www.taylorfrancis.com/books/mono/10.1201/9780203748725/local-polynomial-modelling-applications-jianqing-fan</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>kernel-density-estimation</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Local polynomial generalization that fixes KDE's boundary bias and extends to covariate-conditional regression. §30.5 Rem 9 name-check; §30.9 Rem 17 forwards kernel regression to formalml.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>DUO2007</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Tarn Duong</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>ks: Kernel Density Estimation and Kernel Discriminant Analysis for Multivariate Data in R</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>2007</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Journal of Statistical Software 21(7): 1–16</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.18637/jss.v021.i07</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>kernel-density-estimation</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>The ks R package reference — de-facto multivariate KDE implementation. §30.10 Rem 21 standard multivariate tool citation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>SCO2015</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>David W. Scott</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Multivariate Density Estimation: Theory, Practice, and Visualization</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>978-0-471-69755-8</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>https://onlinelibrary.wiley.com/doi/book/10.1002/9781118575574</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>kernel-density-estimation</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Multivariate-KDE reference. §30.6 Rem 13 cites Ch. 6 for the multivariate AMISE rate O(n^{-4/(4+d)}) — the curse of dimensionality. §30.10 Rem 21 forward-pointer.</t>
         </is>
       </c>
     </row>

</xml_diff>